<commit_message>
Corregir el estandar de malla: 1 cada 2 m de avance
El estandar de la malla no va por disparo sino por avance: 1 malla cada
2 metros, ancho util ya descontado el traslape de 21 cm entre mallas.
Reemplaza la conversion por area que se habia estimado antes.

Efecto en el mes: la malla pasa de 9.16 a 24 unidades y de S/ 10,538 a
S/ 27,600. El total del consumo del mes sube a S/ 123,424. La malla ahora
entra en PEDIR YA: 9 en stock contra 24 que pide el mes.

Queda pendiente confirmar si 1 malla equivale a 1 JGO del maestro (rollo
de 2.42 x 25 m) o a un paño cortado del rollo.

Verificado: 8,323 formulas, 0 errores, las 24 comprobaciones de los 4
materiales coinciden con el desarrollo hecho a mano.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KofGASuDqP2DkSsvGxsHDK
</commit_message>
<xml_diff>
--- a/MRP_ATMIN_corrida_ejemplo_mes.xlsx
+++ b/MRP_ATMIN_corrida_ejemplo_mes.xlsx
@@ -1507,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1683,16 +1683,16 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>rollo 2.42x25 m — ver conversion</t>
+          <t>1 malla cada 2 m de avance (traslape 21 cm)</t>
         </is>
       </c>
       <c r="H9" s="86">
-        <f>(3.5+3.5+3.5)*1.1/(2.42*25)</f>
-        <v/>
-      </c>
-      <c r="I9" s="88" t="inlineStr">
-        <is>
-          <t>SUPUESTO</t>
+        <f>1/2</f>
+        <v/>
+      </c>
+      <c r="I9" s="87" t="inlineStr">
+        <is>
+          <t>DATO REAL</t>
         </is>
       </c>
     </row>
@@ -2303,48 +2303,74 @@
     <row r="40" ht="32" customHeight="1">
       <c r="B40" s="102" t="inlineStr">
         <is>
-          <t>La malla y la resina aguantan.</t>
+          <t>La malla se repone desde la Semana 2.</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>9 rollos y 1,950 cartuchos cubren el mes con holgura. El MRP recien repone hacia el final del horizonte.</t>
+          <t>9 en stock contra 24 que pide el mes. A razon de 1 malla cada 2 m de avance, el stock alcanza solo para las dos primeras semanas.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="B41" s="102" t="inlineStr">
         <is>
-          <t>Dos estandares estan por confirmar.</t>
+          <t>La resina aguanta todo el horizonte.</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
         <is>
-          <t>La malla, porque el maestro la vende en rollo de 2.42 x 25 m y no en paño: hay que convertir por area. Y la resina, porque asumi 2 cartuchos por perno.</t>
+          <t>1,950 cartuchos contra 704 del mes: no hay que pedir nada en las 8 semanas.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="32" customHeight="1">
       <c r="B42" s="102" t="inlineStr">
         <is>
+          <t>Falta cerrar la unidad de la malla.</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>El estandar (1 cada 2 m) es tuyo, pero el maestro la vende como rollo de 2.42 x 25 m. Hay que confirmar si 1 malla = 1 rollo o un paño cortado. Tambien: 2.42 menos 21 cm de traslape da 2.21 m, no 2.00 m — si el ancho util real es 2.21 m, esta corrida pide 10% de mas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="32" customHeight="1">
+      <c r="B43" s="102" t="inlineStr">
+        <is>
+          <t>La resina es un supuesto mio.</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Asumi 2 cartuchos por perno helicoidal. Confirmar cuantos usa realmente cada perno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="B44" s="102" t="inlineStr">
+        <is>
           <t>Faltan precios y lead times.</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>El maestro no los trae. Los que puse son referenciales (naranja). Sin ellos el MRP calcula cantidades correctas pero no fechas de pedido ni costos reales.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="15">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B19:J19"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B28:J28"/>
+    <mergeCell ref="C43:J43"/>
     <mergeCell ref="B36:J36"/>
     <mergeCell ref="C38:J38"/>
     <mergeCell ref="C42:J42"/>
+    <mergeCell ref="C44:J44"/>
     <mergeCell ref="C41:J41"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="A2:J2"/>
@@ -5795,12 +5821,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="51" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>CRNE (Cortada Noreste)</t>
         </is>
       </c>
-      <c r="B6" s="52" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>10-02-90-0006</t>
         </is>
@@ -5813,13 +5839,13 @@
         <f>IFERROR(INDEX(Materiales!$C$4:$C$66,MATCH("#"&amp;$B6,Materiales!$L$4:$L$66,0)),"")</f>
         <v/>
       </c>
-      <c r="E6" s="106">
-        <f>(3.5+3.5+3.5)*1.1/(2.42*25)</f>
-        <v/>
-      </c>
-      <c r="F6" s="37" t="inlineStr">
-        <is>
-          <t>SUPUESTO — el maestro vende la malla en ROLLO de 2.42 x 25 m (60.5 m2), no en paño. Conversion: perimetro 10.5 m (techo + 2 hastiales) x 1.1 de traslape / 60.5 m2 por rollo. CONFIRMAR el perimetro real que se enmalla y el traslape.</t>
+      <c r="E6" s="105">
+        <f>1/2</f>
+        <v/>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>DATO REAL: 1 malla cada 2 m de avance (las mallas traslapan 21 cm entre si)  -&gt;  1 / 2. PENDIENTE: confirmar si 1 malla = 1 JGO del maestro (rollo de 2.42 x 25 m) o un paño cortado del rollo. Ojo: 2.42 - 0.21 de traslape = 2.21 m, no 2.00 m.</t>
         </is>
       </c>
       <c r="G6" s="45">

</xml_diff>

<commit_message>
Escribir la aritmetica real del traslape de la malla en la hoja
El traslape es de 21 cm a cada lado, no a uno solo: 2.42 - 0.21 - 0.21 = 2.00
m de avance por malla, exactos. La celda del estandar ahora lleva la formula
=1/(2.42-2*0.21) en vez de =1/2, para que se vea de donde sale el numero y
se pueda editar si cambia el traslape.

El resultado no cambia (0.5 malla por metro): 24 mallas y S/ 27,600 en el mes.

Verificado: 8,323 formulas, 0 errores, los 5 renglones del bloque de malla
coinciden con el desarrollo hecho a mano.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KofGASuDqP2DkSsvGxsHDK
</commit_message>
<xml_diff>
--- a/MRP_ATMIN_corrida_ejemplo_mes.xlsx
+++ b/MRP_ATMIN_corrida_ejemplo_mes.xlsx
@@ -1683,11 +1683,11 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>1 malla cada 2 m de avance (traslape 21 cm)</t>
+          <t>2.42 m de ancho − 21 cm de traslape a cada lado = 2.00 m de avance por malla</t>
         </is>
       </c>
       <c r="H9" s="86">
-        <f>1/2</f>
+        <f>1/(2.42-2*0.21)</f>
         <v/>
       </c>
       <c r="I9" s="87" t="inlineStr">
@@ -2327,12 +2327,12 @@
     <row r="42" ht="32" customHeight="1">
       <c r="B42" s="102" t="inlineStr">
         <is>
-          <t>Falta cerrar la unidad de la malla.</t>
+          <t>El ancho util de la malla ya esta cerrado.</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>El estandar (1 cada 2 m) es tuyo, pero el maestro la vende como rollo de 2.42 x 25 m. Hay que confirmar si 1 malla = 1 rollo o un paño cortado. Tambien: 2.42 menos 21 cm de traslape da 2.21 m, no 2.00 m — si el ancho util real es 2.21 m, esta corrida pide 10% de mas.</t>
+          <t>2.42 m de ancho menos 21 cm de traslape recortados a cada lado = 2.00 m de avance por malla. Queda una sola duda de unidad: si 1 malla equivale a 1 JGO del maestro o a un paño cortado del rollo de 25 m.</t>
         </is>
       </c>
     </row>
@@ -5840,12 +5840,12 @@
         <v/>
       </c>
       <c r="E6" s="105">
-        <f>1/2</f>
+        <f>1/(2.42-2*0.21)</f>
         <v/>
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>DATO REAL: 1 malla cada 2 m de avance (las mallas traslapan 21 cm entre si)  -&gt;  1 / 2. PENDIENTE: confirmar si 1 malla = 1 JGO del maestro (rollo de 2.42 x 25 m) o un paño cortado del rollo. Ojo: 2.42 - 0.21 de traslape = 2.21 m, no 2.00 m.</t>
+          <t>DATO REAL: la malla mide 2.42 m de ancho y se recortan 21 cm de traslape a CADA lado, asi que cubre 2.42 - 0.21 - 0.21 = 2.00 m de avance  -&gt;  1 malla cada 2 m. Si cambia el traslape, edita la formula de esta celda.</t>
         </is>
       </c>
       <c r="G6" s="45">

</xml_diff>